<commit_message>
Refactor execution substrates for improved directory management and in-memory context handling
- Updated `take-test.sh` and `inject-substrate.sh` scripts to support domain-scoped directories for answer keys and testing data, enhancing flexibility in testing environments.
- Modified `Compat.cs` to utilize reflection for dynamic entity management in the in-memory context, allowing for a more generic handling of entities without hardcoding.
- Enhanced `EffortlessEntityFrameworkRunner.csproj` to streamline the compilation process and exclude generated context files, ensuring cleaner builds.
- Improved documentation and comments across various files to clarify the purpose and functionality of changes, promoting better understanding and maintainability.
</commit_message>
<xml_diff>
--- a/rulebook-examples/acme-llc/effortless-xlsx/ACME, LLC (template).xlsx
+++ b/rulebook-examples/acme-llc/effortless-xlsx/ACME, LLC (template).xlsx
@@ -1,113 +1,92 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eejai42/effortlessapi-app-root/users/user_ee42ai73-18a9-47d5-8f99-954b00f6c041/my-projects/effortlessly-invariant-rulesbooks/rulebook-examples/acme-llc/effortless-xlsx/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989D9A55-649C-8942-A433-E5780F0BA1CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
     <sheet name="Customers" sheetId="1" r:id="rId1"/>
-    <sheet name="ERBVersions" sheetId="2" r:id="rId2"/>
-    <sheet name="ERBCustomizations" sheetId="3" r:id="rId3"/>
-    <sheet name="_original_json" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="ERBVersions" sheetId="2" r:id="rId3"/>
+    <sheet name="ERBCustomizations" sheetId="3" r:id="rId4"/>
+    <sheet name="_original_json" sheetId="4" r:id="rId5" state="hidden"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Customers!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">ERBCustomizations!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">ERBVersions!$A$1:$G$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>CMCC</author>
+    <d:author xmlns:d="http://schemas.openxmlformats.org/spreadsheetml/2006/main">CMCC</d:author>
   </authors>
   <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="B1" authorId="0">
       <text>
         <r>
           <rPr>
+            <rFont val="Aptos Narrow"/>
             <b/>
+            <color rgb="FFFFFFFF"/>
             <sz val="11"/>
-            <color rgb="FFFFFFFF"/>
-            <rFont val="Aptos Narrow"/>
           </rPr>
           <t>Identifier for the customers.</t>
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
+            <rFont val="Aptos Narrow"/>
             <b/>
+            <color rgb="FFFFFFFF"/>
             <sz val="11"/>
-            <color rgb="FFFFFFFF"/>
-            <rFont val="Aptos Narrow"/>
-          </rPr>
-          <t>Thec ustomers email address</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="11"/>
-            <color rgb="FFFFFFFF"/>
-            <rFont val="Aptos Narrow"/>
           </rPr>
           <t>First Name of the customer - used to make the full name</t>
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
+            <rFont val="Aptos Narrow"/>
             <b/>
+            <color rgb="FFFFFFFF"/>
             <sz val="11"/>
-            <color rgb="FFFFFFFF"/>
-            <rFont val="Aptos Narrow"/>
           </rPr>
           <t>Last Name of the customer - used to make the full name</t>
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
+            <rFont val="Aptos Narrow"/>
             <b/>
+            <color rgb="FFFFFFFF"/>
             <sz val="11"/>
-            <color rgb="FFFFFFFF"/>
-            <rFont val="Aptos Narrow"/>
           </rPr>
           <t>Full name is computed from the first and last name of the customer</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <rFont val="Aptos Narrow"/>
+            <b/>
+            <color rgb="FFFFFFFF"/>
+            <sz val="11"/>
+          </rPr>
+          <t>Thec ustomers email address</t>
         </r>
       </text>
     </comment>
@@ -116,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>CustomerId</t>
   </si>
@@ -140,6 +119,9 @@
   </si>
   <si>
     <t>jane.smith@email.com</t>
+  </si>
+  <si>
+    <t>Bobby</t>
   </si>
   <si>
     <t>Smith</t>
@@ -351,7 +333,7 @@
     <t>Data</t>
   </si>
   <si>
-    <t>{
+    <t xml:space="preserve">{
   "$schema": "https://example.com/cmcc-schema/v1",
   "Name": "ACME, LLC (template)",
   "Description": "Rulebook generated from Airtable base \u0027ACME, LLC (template)\u0027.",
@@ -580,15 +562,13 @@
   }
 }</t>
   </si>
-  <si>
-    <t>Bob</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
@@ -633,357 +613,35 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" applyFont="1" fillId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="6" width="17.5" customWidth="1"/>
+    <col min="1" max="1" width="23.053359985351562" customWidth="1"/>
+    <col min="2" max="2" width="22.821292877197266" customWidth="1"/>
+    <col min="3" max="3" width="23.963666915893555" customWidth="1"/>
+    <col min="4" max="4" width="17.443378448486328" customWidth="1"/>
+    <col min="5" max="5" width="17.443378448486328" customWidth="1"/>
+    <col min="6" max="6" width="17.443378448486328" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1003,7 +661,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1015,54 +673,54 @@
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="3" t="str">
         <f>E2 &amp; ", " &amp; D2</f>
-        <v>Smith, Bob</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>Smith, Bobby</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3" t="str">
         <f>SUBSTITUTE(C3, "@", "-")</f>
         <v>john.doe-email.com</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" s="3" t="str">
         <f>E3 &amp; ", " &amp; D3</f>
         <v>Doe, Jimmy</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4" s="3" t="str">
         <f>SUBSTITUTE(C4, "@", "-")</f>
         <v>emily.jones-email.com</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" s="3" t="str">
         <f>E4 &amp; ", " &amp; D4</f>
@@ -1070,198 +728,210 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:F1"/>
+  <headerFooter/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="7" width="17.5" customWidth="1"/>
+    <col min="1" max="1" width="17.443378448486328" customWidth="1"/>
+    <col min="2" max="2" width="17.443378448486328" customWidth="1"/>
+    <col min="3" max="3" width="17.443378448486328" customWidth="1"/>
+    <col min="4" max="4" width="17.443378448486328" customWidth="1"/>
+    <col min="5" max="5" width="17.443378448486328" customWidth="1"/>
+    <col min="6" max="6" width="17.443378448486328" customWidth="1"/>
+    <col min="7" max="7" width="17.443378448486328" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:G1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="27.1640625" customWidth="1"/>
-    <col min="3" max="3" width="34.83203125" customWidth="1"/>
+    <col min="1" max="1" width="27.250761032104492" customWidth="1"/>
+    <col min="2" max="2" width="27.14027214050293" customWidth="1"/>
+    <col min="3" max="3" width="34.911231994628906" customWidth="1"/>
     <col min="4" max="4" width="256" customWidth="1"/>
-    <col min="5" max="5" width="17.5" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" customWidth="1"/>
+    <col min="5" max="5" width="17.443378448486328" customWidth="1"/>
+    <col min="6" max="6" width="19.331968307495117" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="F3" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <autoFilter ref="A1:F1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>54</v>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
+</file>
+
+<file path=EPPlusLicense.txt>This workbook was created with the EPPlus library, licensed to EffortlessAPI Tool under the Polyform Noncommercial license, see https://polyformproject.org/licenses/noncommercial/1.0.0
+For more information about EPPlus, see https://epplussoftware.com/
+
 </file>
</xml_diff>

<commit_message>
acme-llc: clean build, mark ✅ in plan
effortless build runs all transpilers (postgres SQL gen, python,
golang, xlsx, entity-framework, explain-dag, etc.) with exit 0
and no errors. No init-db.sh step, so no Postgres DB side effect.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rulebook-examples/acme-llc/effortless-xlsx/ACME, LLC (template).xlsx
+++ b/rulebook-examples/acme-llc/effortless-xlsx/ACME, LLC (template).xlsx
@@ -543,7 +543,7 @@
     ]
   },
   "_meta": {
-    "_CMCC_Summary": "Airtable export with schema-first type mapping: Schemas, Data, Relationships (FK links), Lookups (INDEX/MATCH), Aggregations (SUMIFS/COUNTIFS/Rollups), and Calculated fields (formulas) in Excel dialect. Field types are determined from Airtable\u0027s schema metadata FIRST (no coercion), with intelligent fallback to formula/data analysis only when schema is unavailable.",
+    "_CMCC_Summary": "Airtable export with schema-first type mapping: Schemas, Data, Relationships (FK links), Lookups (INDEX/MATCH), Aggregations (SUMIFS/COUNTIFS/Rollups), and Calculated fields (formulas) in Excel dialect. Field types are determined from Airtable\u0027s schema metadata FIRST (no coercion); the build FAILS if metadata is unavailable rather than silently inferring from formula/data analysis.",
     "_conversion_metadata": {
       "source_base_id": "appWrXPvXbkgQGOxt",
       "table_count": 3,
@@ -552,9 +552,9 @@
       "export_mode": "schema_first_type_mapping",
       "type_inference": {
         "enabled": true,
-        "priority": "airtable_metadata (NO COERCION) \u2192 formula_analysis \u2192 reference_resolution \u2192 data_analysis (fallback only)",
+        "priority": "airtable_metadata (NO COERCION) \u2192 formula_analysis \u2192 reference_resolution \u2192 data_analysis (last-resort inference; build SHOULD FAIL rather than silently use this)",
         "airtable_type_mapping": "checkbox\u2192boolean, singleLineText\u2192string, multilineText\u2192string, number\u2192number/integer, datetime\u2192datetime, singleSelect\u2192string, email\u2192string, url\u2192string, phoneNumber\u2192string",
-        "data_coercion_hierarchy": "Only used as fallback when Airtable schema unavailable: datetime \u2192 number \u2192 integer \u2192 boolean \u2192 base64 \u2192 json \u2192 string",
+        "data_coercion_hierarchy": "Only invoked when Airtable schema is unavailable (which SHOULD make the build fail). Coercion order: datetime \u2192 number \u2192 integer \u2192 boolean \u2192 base64 \u2192 json \u2192 string",
         "nullable_support": true,
         "error_value_handling": "#NUM!, #ERROR!, #N/A, #REF!, #DIV/0!, #VALUE!, #NAME? are treated as NULL"
       }

</xml_diff>